<commit_message>
Actualizacion de factores ambientales (personal Full-time)
</commit_message>
<xml_diff>
--- a/EstimacionCasosUsos.xlsx
+++ b/EstimacionCasosUsos.xlsx
@@ -1,11 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30121"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7DA6FC0E-18F4-4AC5-9C81-DB91C7A9858F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jmora\Documents\UBP\IS-2\2026\isii\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C37D0B83-F302-457B-9F93-2BFD30B81C7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="4" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CriterioBasadoClasesAnalisis" sheetId="1" r:id="rId1"/>
@@ -508,7 +513,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -841,44 +846,44 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1722,20 +1727,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C18"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.28515625" customWidth="1"/>
     <col min="2" max="2" width="127.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" s="44" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="48" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-    </row>
-    <row r="2" spans="1:3">
+      <c r="B1" s="48"/>
+      <c r="C1" s="48"/>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -1746,7 +1751,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>4</v>
       </c>
@@ -1757,7 +1762,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>6</v>
       </c>
@@ -1768,7 +1773,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>8</v>
       </c>
@@ -1779,19 +1784,19 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
     </row>
-    <row r="8" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A8" s="45" t="s">
+    <row r="8" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="49" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="45"/>
-      <c r="C8" s="45"/>
-    </row>
-    <row r="9" spans="1:3">
+      <c r="B8" s="49"/>
+      <c r="C8" s="49"/>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="3"/>
       <c r="B9" s="4" t="s">
         <v>11</v>
@@ -1800,7 +1805,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>12</v>
       </c>
@@ -1811,7 +1816,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="1:3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>4</v>
       </c>
@@ -1822,7 +1827,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>6</v>
       </c>
@@ -1833,7 +1838,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>8</v>
       </c>
@@ -1844,7 +1849,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="15.75" customHeight="1">
+    <row r="14" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="5"/>
       <c r="B14" s="6" t="s">
         <v>17</v>
@@ -1853,7 +1858,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>12</v>
       </c>
@@ -1864,7 +1869,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="16" spans="1:3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>4</v>
       </c>
@@ -1875,7 +1880,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="1:3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>6</v>
       </c>
@@ -1886,7 +1891,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="18" spans="1:3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>8</v>
       </c>
@@ -1910,7 +1915,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G127"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="48.85546875" customWidth="1"/>
     <col min="2" max="3" width="17.140625" customWidth="1"/>
@@ -1918,15 +1923,15 @@
     <col min="6" max="6" width="17.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="8"/>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>22</v>
       </c>
@@ -1935,7 +1940,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="30.75" customHeight="1">
+    <row r="4" spans="1:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="46" t="s">
         <v>23</v>
       </c>
@@ -1953,7 +1958,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:7">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="40" t="s">
         <v>25</v>
       </c>
@@ -1970,8 +1975,8 @@
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="15">
-      <c r="A6" s="53" t="s">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="43" t="s">
         <v>29</v>
       </c>
       <c r="B6" s="39">
@@ -1988,8 +1993,8 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="15">
-      <c r="A7" s="53" t="s">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="43" t="s">
         <v>31</v>
       </c>
       <c r="B7" s="39">
@@ -2006,8 +2011,8 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="15">
-      <c r="A8" s="53" t="s">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="43" t="s">
         <v>33</v>
       </c>
       <c r="B8" s="39">
@@ -2023,8 +2028,8 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="15">
-      <c r="A9" s="53" t="s">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="43" t="s">
         <v>36</v>
       </c>
       <c r="B9" s="39">
@@ -2041,8 +2046,8 @@
         <v>3</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="15">
-      <c r="A10" s="53" t="s">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="43" t="s">
         <v>38</v>
       </c>
       <c r="B10" s="39">
@@ -2059,8 +2064,8 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="15">
-      <c r="A11" s="53" t="s">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="43" t="s">
         <v>40</v>
       </c>
       <c r="B11" s="39">
@@ -2076,8 +2081,8 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="15">
-      <c r="A12" s="53" t="s">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" s="43" t="s">
         <v>43</v>
       </c>
       <c r="B12" s="39">
@@ -2090,8 +2095,8 @@
       <c r="E12" s="16"/>
       <c r="F12" s="16"/>
     </row>
-    <row r="13" spans="1:7" ht="15">
-      <c r="A13" s="53" t="s">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" s="43" t="s">
         <v>44</v>
       </c>
       <c r="B13" s="39">
@@ -2104,8 +2109,8 @@
       <c r="E13" s="16"/>
       <c r="F13" s="16"/>
     </row>
-    <row r="14" spans="1:7" ht="15">
-      <c r="A14" s="53" t="s">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="43" t="s">
         <v>45</v>
       </c>
       <c r="B14" s="39">
@@ -2114,8 +2119,8 @@
       <c r="E14" s="16"/>
       <c r="F14" s="16"/>
     </row>
-    <row r="15" spans="1:7" ht="15">
-      <c r="A15" s="53" t="s">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" s="43" t="s">
         <v>46</v>
       </c>
       <c r="B15" s="39">
@@ -2125,8 +2130,8 @@
       <c r="E15" s="16"/>
       <c r="F15" s="16"/>
     </row>
-    <row r="16" spans="1:7" ht="15">
-      <c r="A16" s="53" t="s">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="43" t="s">
         <v>47</v>
       </c>
       <c r="B16" s="39">
@@ -2136,8 +2141,8 @@
       <c r="E16" s="16"/>
       <c r="F16" s="16"/>
     </row>
-    <row r="17" spans="1:6" ht="15">
-      <c r="A17" s="53" t="s">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="43" t="s">
         <v>48</v>
       </c>
       <c r="B17" s="39">
@@ -2147,8 +2152,8 @@
       <c r="E17" s="16"/>
       <c r="F17" s="16"/>
     </row>
-    <row r="18" spans="1:6" ht="15">
-      <c r="A18" s="53" t="s">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" s="43" t="s">
         <v>49</v>
       </c>
       <c r="B18" s="39">
@@ -2158,8 +2163,8 @@
       <c r="E18" s="16"/>
       <c r="F18" s="16"/>
     </row>
-    <row r="19" spans="1:6" ht="15">
-      <c r="A19" s="53" t="s">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" s="43" t="s">
         <v>50</v>
       </c>
       <c r="B19" s="39">
@@ -2169,8 +2174,8 @@
       <c r="E19" s="16"/>
       <c r="F19" s="16"/>
     </row>
-    <row r="20" spans="1:6" ht="15">
-      <c r="A20" s="53" t="s">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" s="43" t="s">
         <v>51</v>
       </c>
       <c r="B20" s="39">
@@ -2180,8 +2185,8 @@
       <c r="E20" s="16"/>
       <c r="F20" s="16"/>
     </row>
-    <row r="21" spans="1:6" ht="15">
-      <c r="A21" s="53" t="s">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" s="43" t="s">
         <v>52</v>
       </c>
       <c r="B21" s="39">
@@ -2191,8 +2196,8 @@
       <c r="E21" s="16"/>
       <c r="F21" s="16"/>
     </row>
-    <row r="22" spans="1:6" ht="15">
-      <c r="A22" s="53" t="s">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" s="43" t="s">
         <v>53</v>
       </c>
       <c r="B22" s="39">
@@ -2202,28 +2207,28 @@
       <c r="E22" s="16"/>
       <c r="F22" s="16"/>
     </row>
-    <row r="23" spans="1:6" ht="15">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="41"/>
       <c r="B23" s="39"/>
       <c r="C23" s="19"/>
       <c r="E23" s="16"/>
       <c r="F23" s="16"/>
     </row>
-    <row r="24" spans="1:6" ht="15">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="41"/>
       <c r="B24" s="39"/>
       <c r="C24" s="19"/>
       <c r="E24" s="16"/>
       <c r="F24" s="16"/>
     </row>
-    <row r="25" spans="1:6" ht="15">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="41"/>
       <c r="B25" s="39"/>
       <c r="C25" s="19"/>
       <c r="E25" s="16"/>
       <c r="F25" s="16"/>
     </row>
-    <row r="26" spans="1:6" ht="15">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="41"/>
       <c r="B26" s="39"/>
       <c r="C26" s="19"/>
@@ -2235,7 +2240,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="27" spans="1:6" ht="15">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="41"/>
       <c r="B27" s="39"/>
       <c r="C27" s="19"/>
@@ -2244,7 +2249,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="28" spans="1:6" ht="15">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="41"/>
       <c r="B28" s="39"/>
       <c r="C28" s="19"/>
@@ -2256,7 +2261,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:6" ht="15">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="41"/>
       <c r="B29" s="39"/>
       <c r="C29" s="19"/>
@@ -2265,7 +2270,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:6" ht="15">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="41"/>
       <c r="B30" s="39"/>
       <c r="C30" s="19"/>
@@ -2277,7 +2282,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="31" spans="1:6" ht="15">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="41"/>
       <c r="B31" s="39"/>
       <c r="C31" s="19"/>
@@ -2286,482 +2291,482 @@
         <v>12</v>
       </c>
     </row>
-    <row r="32" spans="1:6" ht="15">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="41"/>
       <c r="B32" s="39"/>
       <c r="C32" s="19"/>
     </row>
-    <row r="33" spans="1:3" ht="15">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="41"/>
       <c r="B33" s="39"/>
       <c r="C33" s="19"/>
     </row>
-    <row r="34" spans="1:3" ht="15">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="41"/>
       <c r="B34" s="39"/>
       <c r="C34" s="19"/>
     </row>
-    <row r="35" spans="1:3" ht="15">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="41"/>
       <c r="B35" s="39"/>
       <c r="C35" s="19"/>
     </row>
-    <row r="36" spans="1:3" ht="15">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="41"/>
       <c r="B36" s="39"/>
       <c r="C36" s="19"/>
     </row>
-    <row r="37" spans="1:3" ht="15">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" s="41"/>
       <c r="B37" s="39"/>
       <c r="C37" s="19"/>
     </row>
-    <row r="38" spans="1:3" ht="15">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" s="41"/>
       <c r="B38" s="39"/>
       <c r="C38" s="19"/>
     </row>
-    <row r="39" spans="1:3" ht="15">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" s="41"/>
       <c r="B39" s="39"/>
       <c r="C39" s="19"/>
     </row>
-    <row r="40" spans="1:3" ht="15">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" s="41"/>
       <c r="B40" s="39"/>
       <c r="C40" s="19"/>
     </row>
-    <row r="41" spans="1:3" ht="15">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" s="41"/>
       <c r="B41" s="39"/>
       <c r="C41" s="19"/>
     </row>
-    <row r="42" spans="1:3" ht="15">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" s="41"/>
       <c r="B42" s="39"/>
       <c r="C42" s="19"/>
     </row>
-    <row r="43" spans="1:3" ht="15">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" s="41"/>
       <c r="B43" s="39"/>
       <c r="C43" s="19"/>
     </row>
-    <row r="44" spans="1:3" ht="15">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" s="41"/>
       <c r="B44" s="39"/>
       <c r="C44" s="19"/>
     </row>
-    <row r="45" spans="1:3" ht="15">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" s="41"/>
       <c r="B45" s="39"/>
       <c r="C45" s="19"/>
     </row>
-    <row r="46" spans="1:3" ht="15">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" s="41"/>
       <c r="B46" s="39"/>
       <c r="C46" s="19"/>
     </row>
-    <row r="47" spans="1:3" ht="15">
-      <c r="A47" s="54"/>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A47" s="44"/>
       <c r="B47" s="16"/>
       <c r="C47" s="19"/>
     </row>
-    <row r="48" spans="1:3" ht="15">
-      <c r="A48" s="55"/>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A48" s="45"/>
       <c r="B48" s="16"/>
       <c r="C48" s="19"/>
     </row>
-    <row r="49" spans="1:3" ht="15">
-      <c r="A49" s="55"/>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A49" s="45"/>
       <c r="B49" s="16"/>
       <c r="C49" s="19"/>
     </row>
-    <row r="50" spans="1:3" ht="15">
-      <c r="A50" s="55"/>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A50" s="45"/>
       <c r="B50" s="16"/>
       <c r="C50" s="19"/>
     </row>
-    <row r="51" spans="1:3" ht="15">
-      <c r="A51" s="55"/>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A51" s="45"/>
       <c r="B51" s="16"/>
       <c r="C51" s="19"/>
     </row>
-    <row r="52" spans="1:3">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" s="16"/>
       <c r="B52" s="16"/>
       <c r="C52" s="19"/>
     </row>
-    <row r="53" spans="1:3">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" s="16"/>
       <c r="B53" s="16"/>
       <c r="C53" s="19"/>
     </row>
-    <row r="54" spans="1:3">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" s="16"/>
       <c r="B54" s="16"/>
       <c r="C54" s="19"/>
     </row>
-    <row r="55" spans="1:3">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" s="16"/>
       <c r="B55" s="16"/>
       <c r="C55" s="19"/>
     </row>
-    <row r="56" spans="1:3">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" s="16"/>
       <c r="B56" s="16"/>
       <c r="C56" s="19"/>
     </row>
-    <row r="57" spans="1:3">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" s="16"/>
       <c r="B57" s="16"/>
       <c r="C57" s="19"/>
     </row>
-    <row r="58" spans="1:3">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" s="16"/>
       <c r="B58" s="16"/>
       <c r="C58" s="19"/>
     </row>
-    <row r="59" spans="1:3">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" s="16"/>
       <c r="B59" s="16"/>
       <c r="C59" s="19"/>
     </row>
-    <row r="60" spans="1:3">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" s="16"/>
       <c r="B60" s="16"/>
       <c r="C60" s="19"/>
     </row>
-    <row r="61" spans="1:3">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" s="16"/>
       <c r="B61" s="16"/>
       <c r="C61" s="19"/>
     </row>
-    <row r="62" spans="1:3">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" s="16"/>
       <c r="B62" s="16"/>
       <c r="C62" s="19"/>
     </row>
-    <row r="63" spans="1:3">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" s="16"/>
       <c r="B63" s="16"/>
       <c r="C63" s="19"/>
     </row>
-    <row r="64" spans="1:3">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" s="16"/>
       <c r="B64" s="16"/>
       <c r="C64" s="19"/>
     </row>
-    <row r="65" spans="1:3">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" s="16"/>
       <c r="B65" s="16"/>
       <c r="C65" s="19"/>
     </row>
-    <row r="66" spans="1:3">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" s="16"/>
       <c r="B66" s="16"/>
       <c r="C66" s="19"/>
     </row>
-    <row r="67" spans="1:3">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" s="16"/>
       <c r="B67" s="16"/>
       <c r="C67" s="19"/>
     </row>
-    <row r="68" spans="1:3">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" s="16"/>
       <c r="B68" s="16"/>
       <c r="C68" s="19"/>
     </row>
-    <row r="69" spans="1:3">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" s="16"/>
       <c r="B69" s="16"/>
       <c r="C69" s="19"/>
     </row>
-    <row r="70" spans="1:3">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" s="16"/>
       <c r="B70" s="16"/>
       <c r="C70" s="19"/>
     </row>
-    <row r="71" spans="1:3">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" s="16"/>
       <c r="B71" s="16"/>
       <c r="C71" s="19"/>
     </row>
-    <row r="72" spans="1:3">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" s="16"/>
       <c r="B72" s="16"/>
       <c r="C72" s="19"/>
     </row>
-    <row r="73" spans="1:3">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" s="16"/>
       <c r="B73" s="16"/>
       <c r="C73" s="19"/>
     </row>
-    <row r="74" spans="1:3">
+    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" s="16"/>
       <c r="B74" s="16"/>
       <c r="C74" s="19"/>
     </row>
-    <row r="75" spans="1:3">
+    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" s="16"/>
       <c r="B75" s="16"/>
       <c r="C75" s="19"/>
     </row>
-    <row r="76" spans="1:3">
+    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76" s="16"/>
       <c r="B76" s="16"/>
       <c r="C76" s="19"/>
     </row>
-    <row r="77" spans="1:3">
+    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A77" s="16"/>
       <c r="B77" s="16"/>
       <c r="C77" s="19"/>
     </row>
-    <row r="78" spans="1:3">
+    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A78" s="16"/>
       <c r="B78" s="16"/>
       <c r="C78" s="19"/>
     </row>
-    <row r="79" spans="1:3">
+    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A79" s="16"/>
       <c r="B79" s="16"/>
       <c r="C79" s="19"/>
     </row>
-    <row r="80" spans="1:3">
+    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A80" s="16"/>
       <c r="B80" s="16"/>
       <c r="C80" s="19"/>
     </row>
-    <row r="81" spans="1:3">
+    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A81" s="16"/>
       <c r="B81" s="16"/>
       <c r="C81" s="19"/>
     </row>
-    <row r="82" spans="1:3">
+    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A82" s="16"/>
       <c r="B82" s="16"/>
       <c r="C82" s="19"/>
     </row>
-    <row r="83" spans="1:3">
+    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A83" s="16"/>
       <c r="B83" s="16"/>
       <c r="C83" s="19"/>
     </row>
-    <row r="84" spans="1:3">
+    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A84" s="16"/>
       <c r="B84" s="16"/>
       <c r="C84" s="19"/>
     </row>
-    <row r="85" spans="1:3">
+    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A85" s="16"/>
       <c r="B85" s="16"/>
       <c r="C85" s="19"/>
     </row>
-    <row r="86" spans="1:3">
+    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A86" s="16"/>
       <c r="B86" s="16"/>
       <c r="C86" s="19"/>
     </row>
-    <row r="87" spans="1:3">
+    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A87" s="16"/>
       <c r="B87" s="16"/>
       <c r="C87" s="19"/>
     </row>
-    <row r="88" spans="1:3">
+    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A88" s="16"/>
       <c r="B88" s="16"/>
       <c r="C88" s="19"/>
     </row>
-    <row r="89" spans="1:3">
+    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A89" s="16"/>
       <c r="B89" s="16"/>
       <c r="C89" s="19"/>
     </row>
-    <row r="90" spans="1:3">
+    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A90" s="16"/>
       <c r="B90" s="16"/>
       <c r="C90" s="19"/>
     </row>
-    <row r="91" spans="1:3">
+    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A91" s="16"/>
       <c r="B91" s="16"/>
       <c r="C91" s="19"/>
     </row>
-    <row r="92" spans="1:3">
+    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A92" s="16"/>
       <c r="B92" s="16"/>
       <c r="C92" s="19"/>
     </row>
-    <row r="93" spans="1:3">
+    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A93" s="16"/>
       <c r="B93" s="16"/>
       <c r="C93" s="19"/>
     </row>
-    <row r="94" spans="1:3">
+    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A94" s="16"/>
       <c r="B94" s="16"/>
       <c r="C94" s="19"/>
     </row>
-    <row r="95" spans="1:3">
+    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A95" s="16"/>
       <c r="B95" s="16"/>
       <c r="C95" s="19"/>
     </row>
-    <row r="96" spans="1:3">
+    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A96" s="16"/>
       <c r="B96" s="16"/>
       <c r="C96" s="19"/>
     </row>
-    <row r="97" spans="1:3">
+    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A97" s="16"/>
       <c r="B97" s="16"/>
       <c r="C97" s="19"/>
     </row>
-    <row r="98" spans="1:3">
+    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A98" s="16"/>
       <c r="B98" s="16"/>
       <c r="C98" s="19"/>
     </row>
-    <row r="99" spans="1:3">
+    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A99" s="16"/>
       <c r="B99" s="16"/>
       <c r="C99" s="19"/>
     </row>
-    <row r="100" spans="1:3">
+    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A100" s="16"/>
       <c r="B100" s="16"/>
       <c r="C100" s="19"/>
     </row>
-    <row r="101" spans="1:3">
+    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A101" s="16"/>
       <c r="B101" s="16"/>
       <c r="C101" s="19"/>
     </row>
-    <row r="102" spans="1:3">
+    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A102" s="16"/>
       <c r="B102" s="16"/>
       <c r="C102" s="19"/>
     </row>
-    <row r="103" spans="1:3">
+    <row r="103" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A103" s="16"/>
       <c r="B103" s="16"/>
       <c r="C103" s="19"/>
     </row>
-    <row r="104" spans="1:3">
+    <row r="104" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A104" s="16"/>
       <c r="B104" s="16"/>
       <c r="C104" s="19"/>
     </row>
-    <row r="105" spans="1:3">
+    <row r="105" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A105" s="16"/>
       <c r="B105" s="16"/>
       <c r="C105" s="19"/>
     </row>
-    <row r="106" spans="1:3">
+    <row r="106" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A106" s="16"/>
       <c r="B106" s="16"/>
       <c r="C106" s="19"/>
     </row>
-    <row r="107" spans="1:3">
+    <row r="107" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A107" s="16"/>
       <c r="B107" s="16"/>
       <c r="C107" s="19"/>
     </row>
-    <row r="108" spans="1:3">
+    <row r="108" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A108" s="16"/>
       <c r="B108" s="16"/>
       <c r="C108" s="19"/>
     </row>
-    <row r="109" spans="1:3">
+    <row r="109" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A109" s="16"/>
       <c r="B109" s="16"/>
       <c r="C109" s="19"/>
     </row>
-    <row r="110" spans="1:3">
+    <row r="110" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A110" s="16"/>
       <c r="B110" s="16"/>
       <c r="C110" s="19"/>
     </row>
-    <row r="111" spans="1:3">
+    <row r="111" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A111" s="16"/>
       <c r="B111" s="16"/>
       <c r="C111" s="19"/>
     </row>
-    <row r="112" spans="1:3">
+    <row r="112" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A112" s="16"/>
       <c r="B112" s="16"/>
       <c r="C112" s="19"/>
     </row>
-    <row r="113" spans="1:3">
+    <row r="113" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A113" s="16"/>
       <c r="B113" s="16"/>
       <c r="C113" s="19"/>
     </row>
-    <row r="114" spans="1:3">
+    <row r="114" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A114" s="16"/>
       <c r="B114" s="16"/>
       <c r="C114" s="19"/>
     </row>
-    <row r="115" spans="1:3">
+    <row r="115" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A115" s="16"/>
       <c r="B115" s="16"/>
       <c r="C115" s="19"/>
     </row>
-    <row r="116" spans="1:3">
+    <row r="116" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A116" s="16"/>
       <c r="B116" s="16"/>
       <c r="C116" s="19"/>
     </row>
-    <row r="117" spans="1:3">
+    <row r="117" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A117" s="16"/>
       <c r="B117" s="16"/>
       <c r="C117" s="19"/>
     </row>
-    <row r="118" spans="1:3">
+    <row r="118" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A118" s="16"/>
       <c r="B118" s="16"/>
       <c r="C118" s="19"/>
     </row>
-    <row r="119" spans="1:3">
+    <row r="119" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A119" s="16"/>
       <c r="B119" s="16"/>
       <c r="C119" s="19"/>
     </row>
-    <row r="120" spans="1:3">
+    <row r="120" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A120" s="16"/>
       <c r="B120" s="16"/>
       <c r="C120" s="19"/>
     </row>
-    <row r="121" spans="1:3">
+    <row r="121" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A121" s="16"/>
       <c r="B121" s="16"/>
       <c r="C121" s="19"/>
     </row>
-    <row r="122" spans="1:3">
+    <row r="122" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A122" s="16"/>
       <c r="B122" s="16"/>
       <c r="C122" s="19"/>
     </row>
-    <row r="123" spans="1:3">
+    <row r="123" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A123" s="16"/>
       <c r="B123" s="16"/>
       <c r="C123" s="19"/>
     </row>
-    <row r="124" spans="1:3">
+    <row r="124" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A124" s="16"/>
       <c r="B124" s="16"/>
       <c r="C124" s="19"/>
     </row>
-    <row r="125" spans="1:3">
+    <row r="125" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A125" s="16"/>
       <c r="B125" s="16"/>
       <c r="C125" s="19"/>
     </row>
-    <row r="126" spans="1:3">
+    <row r="126" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A126" s="16"/>
       <c r="B126" s="16"/>
       <c r="C126" s="19"/>
     </row>
-    <row r="127" spans="1:3">
+    <row r="127" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A127" s="16"/>
       <c r="B127" s="16"/>
       <c r="C127" s="19"/>
@@ -2819,7 +2824,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:J29"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="57.85546875" customWidth="1"/>
     <col min="4" max="5" width="9.85546875" customWidth="1"/>
@@ -2829,22 +2834,22 @@
     <col min="10" max="10" width="8.28515625" style="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="14.25" customHeight="1">
-      <c r="A1" s="48" t="s">
+    <row r="1" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="50" t="s">
         <v>57</v>
       </c>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
+      <c r="B1" s="50"/>
+      <c r="C1" s="50"/>
       <c r="D1" s="21">
         <f>0.6+(0.01*SUM(E3:E15))</f>
         <v>0.96499999999999997</v>
       </c>
-      <c r="I1" s="49" t="s">
+      <c r="I1" s="51" t="s">
         <v>58</v>
       </c>
-      <c r="J1" s="49"/>
-    </row>
-    <row r="2" spans="1:10">
+      <c r="J1" s="51"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="22" t="s">
         <v>59</v>
       </c>
@@ -2861,10 +2866,10 @@
         <v>62</v>
       </c>
       <c r="F2" s="24"/>
-      <c r="I2" s="49"/>
-      <c r="J2" s="49"/>
-    </row>
-    <row r="3" spans="1:10">
+      <c r="I2" s="51"/>
+      <c r="J2" s="51"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>63</v>
       </c>
@@ -2878,7 +2883,7 @@
         <v>2</v>
       </c>
       <c r="E3" s="2">
-        <f>C3*D3</f>
+        <f t="shared" ref="E3:E15" si="0">C3*D3</f>
         <v>4</v>
       </c>
       <c r="I3" s="26" t="s">
@@ -2888,7 +2893,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="29.25" customHeight="1">
+    <row r="4" spans="1:10" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="28" t="s">
         <v>66</v>
       </c>
@@ -2902,7 +2907,7 @@
         <v>3</v>
       </c>
       <c r="E4" s="2">
-        <f>C4*D4</f>
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
       <c r="I4" s="2" t="s">
@@ -2912,7 +2917,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="5" spans="1:10">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>70</v>
       </c>
@@ -2926,7 +2931,7 @@
         <v>4</v>
       </c>
       <c r="E5" s="2">
-        <f>C5*D5</f>
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="I5" s="2" t="s">
@@ -2936,7 +2941,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="6" spans="1:10">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>73</v>
       </c>
@@ -2950,7 +2955,7 @@
         <v>4</v>
       </c>
       <c r="E6" s="2">
-        <f>C6*D6</f>
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="I6" s="2" t="s">
@@ -2960,7 +2965,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:10">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>76</v>
       </c>
@@ -2974,11 +2979,11 @@
         <v>2</v>
       </c>
       <c r="E7" s="2">
-        <f>C7*D7</f>
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:10">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>78</v>
       </c>
@@ -2992,11 +2997,11 @@
         <v>3</v>
       </c>
       <c r="E8" s="2">
-        <f>C8*D8</f>
+        <f t="shared" si="0"/>
         <v>1.5</v>
       </c>
     </row>
-    <row r="9" spans="1:10">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>80</v>
       </c>
@@ -3010,11 +3015,11 @@
         <v>4</v>
       </c>
       <c r="E9" s="2">
-        <f>C9*D9</f>
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="1:10">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>82</v>
       </c>
@@ -3028,11 +3033,11 @@
         <v>1</v>
       </c>
       <c r="E10" s="2">
-        <f>C10*D10</f>
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:10">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>84</v>
       </c>
@@ -3046,11 +3051,11 @@
         <v>3</v>
       </c>
       <c r="E11" s="2">
-        <f>C11*D11</f>
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:10">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>86</v>
       </c>
@@ -3064,11 +3069,11 @@
         <v>3</v>
       </c>
       <c r="E12" s="2">
-        <f>C12*D12</f>
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="1:10">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>88</v>
       </c>
@@ -3082,11 +3087,11 @@
         <v>3</v>
       </c>
       <c r="E13" s="2">
-        <f>C13*D13</f>
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="1:10">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>90</v>
       </c>
@@ -3100,11 +3105,11 @@
         <v>4</v>
       </c>
       <c r="E14" s="2">
-        <f>C14*D14</f>
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="1:10">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>92</v>
       </c>
@@ -3118,31 +3123,31 @@
         <v>1</v>
       </c>
       <c r="E15" s="2">
-        <f>C15*D15</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="17.25" customHeight="1">
-      <c r="A16" s="50" t="s">
+    <row r="16" spans="1:10" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="52" t="s">
         <v>94</v>
       </c>
-      <c r="B16" s="50"/>
-      <c r="C16" s="50"/>
+      <c r="B16" s="52"/>
+      <c r="C16" s="52"/>
       <c r="D16" s="21">
         <f>1.4-(0.03*SUM(E18:E25))</f>
-        <v>0.98</v>
-      </c>
-      <c r="G16" s="50" t="s">
+        <v>0.83</v>
+      </c>
+      <c r="G16" s="52" t="s">
         <v>95</v>
       </c>
-      <c r="H16" s="50"/>
-      <c r="I16" s="50"/>
+      <c r="H16" s="52"/>
+      <c r="I16" s="52"/>
       <c r="J16" s="30">
         <f>'PCU-Ajustado'!C3*IF(I20&lt;=2,20,IF(AND(I20&gt;2,I20&lt;=4),28,36))</f>
-        <v>2534.4760000000001</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9">
+        <v>2146.5459999999998</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="31" t="s">
         <v>3</v>
       </c>
@@ -3169,7 +3174,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="18" spans="1:9">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>98</v>
       </c>
@@ -3183,7 +3188,7 @@
         <v>3</v>
       </c>
       <c r="E18" s="2">
-        <f>C18*D18</f>
+        <f t="shared" ref="E18:E25" si="1">C18*D18</f>
         <v>4.5</v>
       </c>
       <c r="G18" t="s">
@@ -3197,7 +3202,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:9">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>102</v>
       </c>
@@ -3211,7 +3216,7 @@
         <v>2</v>
       </c>
       <c r="E19" s="2">
-        <f>C19*D19</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="G19" t="s">
@@ -3222,10 +3227,10 @@
       </c>
       <c r="I19">
         <f>COUNTIF(D24:D25,"&gt;3")</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>106</v>
       </c>
@@ -3239,7 +3244,7 @@
         <v>3</v>
       </c>
       <c r="E20" s="2">
-        <f>C20*D20</f>
+        <f t="shared" si="1"/>
         <v>3</v>
       </c>
       <c r="H20" s="34" t="s">
@@ -3247,10 +3252,10 @@
       </c>
       <c r="I20" s="34">
         <f>SUM(I18:I19)</f>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>108</v>
       </c>
@@ -3264,16 +3269,16 @@
         <v>3</v>
       </c>
       <c r="E21" s="2">
-        <f>C21*D21</f>
+        <f t="shared" si="1"/>
         <v>1.5</v>
       </c>
-      <c r="G21" s="51" t="s">
+      <c r="G21" s="53" t="s">
         <v>110</v>
       </c>
-      <c r="H21" s="51"/>
-      <c r="I21" s="51"/>
-    </row>
-    <row r="22" spans="1:9">
+      <c r="H21" s="53"/>
+      <c r="I21" s="53"/>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>111</v>
       </c>
@@ -3287,7 +3292,7 @@
         <v>3</v>
       </c>
       <c r="E22" s="2">
-        <f>C22*D22</f>
+        <f t="shared" si="1"/>
         <v>3</v>
       </c>
       <c r="G22" s="35" t="s">
@@ -3297,7 +3302,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="23" spans="1:9">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>114</v>
       </c>
@@ -3311,7 +3316,7 @@
         <v>4</v>
       </c>
       <c r="E23" s="2">
-        <f>C23*D23</f>
+        <f t="shared" si="1"/>
         <v>8</v>
       </c>
       <c r="G23" s="29">
@@ -3321,7 +3326,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="24" spans="1:9">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>117</v>
       </c>
@@ -3332,11 +3337,11 @@
         <v>-1</v>
       </c>
       <c r="D24" s="2">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E24" s="2">
-        <f>C24*D24</f>
-        <v>-5</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
       <c r="G24" s="29">
         <v>28</v>
@@ -3345,7 +3350,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="25" spans="1:9">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>120</v>
       </c>
@@ -3359,7 +3364,7 @@
         <v>2</v>
       </c>
       <c r="E25" s="2">
-        <f>C25*D25</f>
+        <f t="shared" si="1"/>
         <v>-2</v>
       </c>
       <c r="G25" s="29">
@@ -3369,7 +3374,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="27" spans="1:9">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D27">
         <v>1</v>
       </c>
@@ -3377,7 +3382,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="28" spans="1:9">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D28">
         <v>3</v>
       </c>
@@ -3385,7 +3390,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="29" spans="1:9">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D29">
         <v>5</v>
       </c>
@@ -3416,22 +3421,22 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultColWidth="10.7109375" defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:6" ht="71.25" customHeight="1">
-      <c r="A1" s="52" t="s">
+    <row r="1" spans="1:6" ht="71.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="54" t="s">
         <v>126</v>
       </c>
-      <c r="B1" s="52"/>
-      <c r="C1" s="52"/>
-      <c r="D1" s="52"/>
-      <c r="E1" s="52"/>
-      <c r="F1" s="52"/>
-    </row>
-    <row r="3" spans="1:6" ht="19.7">
+      <c r="B1" s="54"/>
+      <c r="C1" s="54"/>
+      <c r="D1" s="54"/>
+      <c r="E1" s="54"/>
+      <c r="F1" s="54"/>
+    </row>
+    <row r="3" spans="1:6" ht="21" x14ac:dyDescent="0.35">
       <c r="C3" s="36">
         <f>'PCU-sinAjustar'!B3*Factores!D1*Factores!D16</f>
-        <v>126.7238</v>
+        <v>107.32729999999999</v>
       </c>
     </row>
   </sheetData>
@@ -3447,7 +3452,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A7:I25"/>
-  <sheetFormatPr defaultColWidth="10.7109375" defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="28" customWidth="1"/>
     <col min="3" max="3" width="12.28515625" customWidth="1"/>
@@ -3455,20 +3460,20 @@
     <col min="5" max="5" width="29.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="7" spans="1:9">
-      <c r="A7" s="43" t="s">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" s="55" t="s">
         <v>127</v>
       </c>
-      <c r="B7" s="43"/>
-      <c r="C7" s="43"/>
-      <c r="D7" s="43"/>
-      <c r="E7" s="43"/>
-      <c r="F7" s="43"/>
-      <c r="G7" s="43"/>
-      <c r="H7" s="43"/>
-      <c r="I7" s="43"/>
-    </row>
-    <row r="9" spans="1:9">
+      <c r="B7" s="55"/>
+      <c r="C7" s="55"/>
+      <c r="D7" s="55"/>
+      <c r="E7" s="55"/>
+      <c r="F7" s="55"/>
+      <c r="G7" s="55"/>
+      <c r="H7" s="55"/>
+      <c r="I7" s="55"/>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B9" s="37" t="s">
         <v>128</v>
       </c>
@@ -3482,7 +3487,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="10" spans="1:9">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B10" s="2" t="s">
         <v>132</v>
       </c>
@@ -3491,14 +3496,14 @@
       </c>
       <c r="D10" s="2">
         <f>($C$10*$D$15)/100</f>
-        <v>950.4285000000001</v>
+        <v>804.95474999999988</v>
       </c>
       <c r="E10" s="2">
         <f>$D$10/8</f>
-        <v>118.80356250000001</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9">
+        <v>100.61934374999998</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B11" s="2" t="s">
         <v>133</v>
       </c>
@@ -3507,14 +3512,14 @@
       </c>
       <c r="D11" s="2">
         <f>($C$11*$D$15)/100</f>
-        <v>1267.2380000000003</v>
+        <v>1073.2729999999999</v>
       </c>
       <c r="E11" s="2">
         <f>$D$11/8</f>
-        <v>158.40475000000004</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9">
+        <v>134.15912499999999</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B12" s="38" t="s">
         <v>134</v>
       </c>
@@ -3523,14 +3528,14 @@
       </c>
       <c r="D12" s="37">
         <f>Factores!$J$16</f>
-        <v>2534.4760000000001</v>
+        <v>2146.5459999999998</v>
       </c>
       <c r="E12" s="38">
         <f>$D$12/8</f>
-        <v>316.80950000000001</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9">
+        <v>268.31824999999998</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B13" s="2" t="s">
         <v>135</v>
       </c>
@@ -3539,14 +3544,14 @@
       </c>
       <c r="D13" s="2">
         <f>($C$13*$D$15)/$C$15</f>
-        <v>1267.2380000000003</v>
+        <v>1073.2729999999999</v>
       </c>
       <c r="E13" s="2">
         <f>$D$13/8</f>
-        <v>158.40475000000004</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9">
+        <v>134.15912499999999</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B14" s="2" t="s">
         <v>136</v>
       </c>
@@ -3555,14 +3560,14 @@
       </c>
       <c r="D14" s="2">
         <f>($C$14*$D$15)/100</f>
-        <v>316.80950000000007</v>
+        <v>268.31824999999998</v>
       </c>
       <c r="E14" s="2">
         <f>$D$14/8</f>
-        <v>39.601187500000009</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9">
+        <v>33.539781249999997</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B15" s="37" t="s">
         <v>97</v>
       </c>
@@ -3572,14 +3577,14 @@
       </c>
       <c r="D15" s="37">
         <f>($C$15*$D$12)/$C$12</f>
-        <v>6336.1900000000005</v>
+        <v>5366.3649999999998</v>
       </c>
       <c r="E15" s="37">
         <f>$D$15/8</f>
-        <v>792.02375000000006</v>
-      </c>
-    </row>
-    <row r="17" spans="2:6">
+        <v>670.79562499999997</v>
+      </c>
+    </row>
+    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B17" s="37" t="s">
         <v>137</v>
       </c>
@@ -3587,39 +3592,39 @@
         <v>138</v>
       </c>
     </row>
-    <row r="18" spans="2:6">
+    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B18" s="21" t="s">
         <v>139</v>
       </c>
       <c r="C18" s="21">
         <f>$D$15/8</f>
-        <v>792.02375000000006</v>
+        <v>670.79562499999997</v>
       </c>
       <c r="E18" s="21" t="s">
         <v>139</v>
       </c>
       <c r="F18" s="21">
         <f>$D$12/8</f>
-        <v>316.80950000000001</v>
-      </c>
-    </row>
-    <row r="19" spans="2:6">
+        <v>268.31824999999998</v>
+      </c>
+    </row>
+    <row r="19" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B19" s="21" t="s">
         <v>140</v>
       </c>
       <c r="C19" s="21">
         <f>$C$18/20</f>
-        <v>39.601187500000002</v>
+        <v>33.539781249999997</v>
       </c>
       <c r="E19" s="21" t="s">
         <v>140</v>
       </c>
       <c r="F19" s="21">
         <f>$F$18/20</f>
-        <v>15.840475000000001</v>
-      </c>
-    </row>
-    <row r="22" spans="2:6" ht="15">
+        <v>13.415912499999999</v>
+      </c>
+    </row>
+    <row r="22" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B22" s="42" t="s">
         <v>141</v>
       </c>
@@ -3627,7 +3632,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="23" spans="2:6" ht="15">
+    <row r="23" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B23" s="37" t="s">
         <v>137</v>
       </c>
@@ -3635,36 +3640,36 @@
         <v>138</v>
       </c>
     </row>
-    <row r="24" spans="2:6" ht="15">
+    <row r="24" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B24" s="21" t="s">
         <v>139</v>
       </c>
       <c r="C24" s="21">
         <f>($D$15/8)/4</f>
-        <v>198.00593750000002</v>
+        <v>167.69890624999999</v>
       </c>
       <c r="E24" s="21" t="s">
         <v>139</v>
       </c>
       <c r="F24" s="21">
         <f>($D$12/8)/4</f>
-        <v>79.202375000000004</v>
-      </c>
-    </row>
-    <row r="25" spans="2:6" ht="15">
+        <v>67.079562499999994</v>
+      </c>
+    </row>
+    <row r="25" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B25" s="21" t="s">
         <v>140</v>
       </c>
       <c r="C25" s="21">
         <f>($C$18/20)/4</f>
-        <v>9.9002968750000004</v>
+        <v>8.3849453124999993</v>
       </c>
       <c r="E25" s="21" t="s">
         <v>140</v>
       </c>
       <c r="F25" s="21">
         <f>($F$18/20)/4</f>
-        <v>3.9601187500000004</v>
+        <v>3.3539781249999998</v>
       </c>
     </row>
   </sheetData>
@@ -3816,5 +3821,19 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D6944D40-E467-4DD6-A6FD-F67719449E45}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D6944D40-E467-4DD6-A6FD-F67719449E45}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="3d2ce1d5-7ded-494d-8056-a72947510cdc"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>